<commit_message>
fix: reforzar seguridad, persistencia y pruebas
</commit_message>
<xml_diff>
--- a/docs/testing/Digital-Money-House-Test-Suites.xlsx
+++ b/docs/testing/Digital-Money-House-Test-Suites.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R6607d240c71f45c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos" sheetId="2" r:id="Rce53dfe931c44073"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="Rb67475a082e04d5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos" sheetId="2" r:id="R16673024ed4646d0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +17,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -58,6 +58,12 @@
       <x:color rgb="FF375623"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F1F1F"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
   <x:fills count="6">
     <x:fill>
@@ -241,7 +247,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="73">
+  <x:cellXfs count="77">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -404,6 +410,18 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -624,9 +642,9 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="62" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -653,10 +671,10 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="24" t="str">
-        <x:v>Fecha de ejecución</x:v>
+        <x:v>Fecha de actualización</x:v>
       </x:c>
       <x:c r="B3" s="25" t="d">
-        <x:v>2026-10-13T00:00:00.000Z</x:v>
+        <x:v>2026-10-21T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C3" s="23"/>
       <x:c r="D3" s="23"/>
@@ -691,13 +709,13 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="26" t="str">
-        <x:v>Suite</x:v>
+        <x:v>Métrica</x:v>
       </x:c>
       <x:c r="B6" s="26" t="str">
-        <x:v>Casos</x:v>
+        <x:v>Cantidad</x:v>
       </x:c>
       <x:c r="C6" s="26" t="str">
-        <x:v>Aprobados</x:v>
+        <x:v>Estado</x:v>
       </x:c>
       <x:c r="D6" s="23"/>
       <x:c r="E6" s="23"/>
@@ -707,15 +725,13 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="27" t="str">
-        <x:v>Smoke</x:v>
+        <x:v>Casos diseñados</x:v>
       </x:c>
       <x:c r="B7" s="28" t="n">
-        <x:f>COUNTIF(Casos!C:C,A7)</x:f>
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C7" s="29" t="n">
-        <x:f>COUNTIFS(Casos!C:C,A7,Casos!H:H,"Aprobado")</x:f>
-        <x:v>2</x:v>
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="C7" s="73" t="str">
+        <x:v>Cobertura manual de Sprint 2, 3 y 4</x:v>
       </x:c>
       <x:c r="D7" s="23"/>
       <x:c r="E7" s="23"/>
@@ -725,15 +741,13 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="30" t="str">
-        <x:v>Regression</x:v>
+        <x:v>Casos ejecutados</x:v>
       </x:c>
       <x:c r="B8" s="31" t="n">
-        <x:f>COUNTIF(Casos!C:C,A8)</x:f>
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C8" s="32" t="n">
-        <x:f>COUNTIFS(Casos!C:C,A8,Casos!H:H,"Aprobado")</x:f>
-        <x:v>12</x:v>
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C8" s="74" t="str">
+        <x:v>14 aprobados</x:v>
       </x:c>
       <x:c r="D8" s="23"/>
       <x:c r="E8" s="23"/>
@@ -742,21 +756,27 @@
       <x:c r="H8" s="23"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="23"/>
-      <x:c r="B9" s="23"/>
-      <x:c r="C9" s="23"/>
+      <x:c r="A9" s="23" t="str">
+        <x:v>Casos pendientes</x:v>
+      </x:c>
+      <x:c r="B9" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C9" s="75" t="str">
+        <x:v>S4-07 a S4-09: ejecutar en Postman</x:v>
+      </x:c>
       <x:c r="D9" s="23"/>
       <x:c r="E9" s="23"/>
       <x:c r="F9" s="23"/>
       <x:c r="G9" s="23"/>
       <x:c r="H9" s="23"/>
     </x:row>
-    <x:row r="10" ht="32" customHeight="1">
-      <x:c r="A10" s="33" t="str">
-        <x:v>Resultado: los casos registrados se ejecutaron satisfactoriamente. Los escenarios de error se verificaron contra la API y los flujos principales en FrontEnd.</x:v>
-      </x:c>
-      <x:c r="B10" s="33"/>
-      <x:c r="C10" s="33"/>
+    <x:row r="10" ht="42" customHeight="1">
+      <x:c r="A10" s="76" t="str">
+        <x:v>Resultado: 14 casos ejecutados y aprobados. S4-07 a S4-09 quedan pendientes de Postman.</x:v>
+      </x:c>
+      <x:c r="B10" s="76"/>
+      <x:c r="C10" s="76"/>
       <x:c r="D10" s="33"/>
       <x:c r="E10" s="33"/>
       <x:c r="F10" s="33"/>
@@ -786,7 +806,6 @@
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A10:H10"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1255,13 +1274,100 @@
         <x:v>Prueba manual 2026-10-13</x:v>
       </x:c>
     </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="61" t="str">
+        <x:v>S4-07</x:v>
+      </x:c>
+      <x:c r="B18" s="62" t="str">
+        <x:v>Sprint 4</x:v>
+      </x:c>
+      <x:c r="C18" s="62" t="str">
+        <x:v>Regression</x:v>
+      </x:c>
+      <x:c r="D18" s="62" t="str">
+        <x:v>API</x:v>
+      </x:c>
+      <x:c r="E18" s="62" t="str">
+        <x:v>Transferencia a cuenta propia</x:v>
+      </x:c>
+      <x:c r="F18" s="62" t="str">
+        <x:v>Enviar una transferencia al alias o CVU de la misma cuenta.</x:v>
+      </x:c>
+      <x:c r="G18" s="62" t="str">
+        <x:v>HTTP 400 y saldo sin cambios.</x:v>
+      </x:c>
+      <x:c r="H18" s="72" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="I18" s="63" t="str">
+        <x:v>Postman: Error: transferencia a cuenta propia</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="61" t="str">
+        <x:v>S4-08</x:v>
+      </x:c>
+      <x:c r="B19" s="62" t="str">
+        <x:v>Sprint 4</x:v>
+      </x:c>
+      <x:c r="C19" s="62" t="str">
+        <x:v>Regression</x:v>
+      </x:c>
+      <x:c r="D19" s="62" t="str">
+        <x:v>API</x:v>
+      </x:c>
+      <x:c r="E19" s="62" t="str">
+        <x:v>Monto de transferencia inválido</x:v>
+      </x:c>
+      <x:c r="F19" s="62" t="str">
+        <x:v>Enviar una transferencia con importe cero o negativo.</x:v>
+      </x:c>
+      <x:c r="G19" s="62" t="str">
+        <x:v>HTTP 400 y sin movimientos.</x:v>
+      </x:c>
+      <x:c r="H19" s="72" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="I19" s="63" t="str">
+        <x:v>Postman: Error: importe inválido</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="61" t="str">
+        <x:v>S4-09</x:v>
+      </x:c>
+      <x:c r="B20" s="62" t="str">
+        <x:v>Sprint 4</x:v>
+      </x:c>
+      <x:c r="C20" s="62" t="str">
+        <x:v>Smoke</x:v>
+      </x:c>
+      <x:c r="D20" s="62" t="str">
+        <x:v>Seguridad</x:v>
+      </x:c>
+      <x:c r="E20" s="62" t="str">
+        <x:v>Transferencia sin token</x:v>
+      </x:c>
+      <x:c r="F20" s="62" t="str">
+        <x:v>Enviar una transferencia sin encabezado Authorization.</x:v>
+      </x:c>
+      <x:c r="G20" s="62" t="str">
+        <x:v>HTTP 401.</x:v>
+      </x:c>
+      <x:c r="H20" s="72" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="I20" s="63" t="str">
+        <x:v>Postman: Error: petición sin token</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:I1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cd8e191692d4fe7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d86d00bf65e4123"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: cerrar evidencia de pruebas sprint 4
</commit_message>
<xml_diff>
--- a/docs/testing/Digital-Money-House-Test-Suites.xlsx
+++ b/docs/testing/Digital-Money-House-Test-Suites.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="Rb67475a082e04d5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos" sheetId="2" r:id="R16673024ed4646d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R6c5588d748cd43b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos" sheetId="2" r:id="Rfbb040031092498a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -688,7 +688,7 @@
         <x:v>Ambiente</x:v>
       </x:c>
       <x:c r="B4" s="23" t="str">
-        <x:v>Gateway localhost:8080, Keycloak, MySQL y FrontEnd localhost:3000</x:v>
+        <x:v>Cloud local: FrontEnd localhost:8088, Gateway, Keycloak y MySQL</x:v>
       </x:c>
       <x:c r="C4" s="23"/>
       <x:c r="D4" s="23"/>
@@ -744,10 +744,10 @@
         <x:v>Casos ejecutados</x:v>
       </x:c>
       <x:c r="B8" s="31" t="n">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C8" s="74" t="str">
-        <x:v>14 aprobados</x:v>
+        <x:v>17 aprobados</x:v>
       </x:c>
       <x:c r="D8" s="23"/>
       <x:c r="E8" s="23"/>
@@ -760,10 +760,10 @@
         <x:v>Casos pendientes</x:v>
       </x:c>
       <x:c r="B9" s="23" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C9" s="75" t="str">
-        <x:v>S4-07 a S4-09: ejecutar en Postman</x:v>
+        <x:v>Sin pendientes</x:v>
       </x:c>
       <x:c r="D9" s="23"/>
       <x:c r="E9" s="23"/>
@@ -773,7 +773,7 @@
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="76" t="str">
-        <x:v>Resultado: 14 casos ejecutados y aprobados. S4-07 a S4-09 quedan pendientes de Postman.</x:v>
+        <x:v>Resultado: 17 casos ejecutados y aprobados. Sin casos pendientes.</x:v>
       </x:c>
       <x:c r="B10" s="76"/>
       <x:c r="C10" s="76"/>
@@ -1297,10 +1297,10 @@
         <x:v>HTTP 400 y saldo sin cambios.</x:v>
       </x:c>
       <x:c r="H18" s="72" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
       <x:c r="I18" s="63" t="str">
-        <x:v>Postman: Error: transferencia a cuenta propia</x:v>
+        <x:v>Postman cloud 2026-10-21 — HTTP 400</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1326,10 +1326,10 @@
         <x:v>HTTP 400 y sin movimientos.</x:v>
       </x:c>
       <x:c r="H19" s="72" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
       <x:c r="I19" s="63" t="str">
-        <x:v>Postman: Error: importe inválido</x:v>
+        <x:v>Postman cloud 2026-10-21 — HTTP 400</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1355,10 +1355,10 @@
         <x:v>HTTP 401.</x:v>
       </x:c>
       <x:c r="H20" s="72" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
       <x:c r="I20" s="63" t="str">
-        <x:v>Postman: Error: petición sin token</x:v>
+        <x:v>Postman cloud 2026-10-21 — HTTP 401</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1367,7 +1367,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d86d00bf65e4123"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refd5572a060a4b5b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>